<commit_message>
Ajout données espèces, export liste espèces parc, amorce comparaison intersecteur
</commit_message>
<xml_diff>
--- a/data/photogrammetrie.xlsx
+++ b/data/photogrammetrie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Andromede\PROJETS\CARHO\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860117E8-6A76-4EC5-A78E-31D60DB1B040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900F4882-176E-4AD6-B2FA-3005D4349F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BA83D1F-2BE6-44A2-8C50-3D2613E4E1D0}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{5BA83D1F-2BE6-44A2-8C50-3D2613E4E1D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="34">
   <si>
     <t>Station</t>
   </si>
@@ -69,12 +69,6 @@
     <t>R_PNMCCA_08</t>
   </si>
   <si>
-    <t>Surface 2D</t>
-  </si>
-  <si>
-    <t>Surface 3D</t>
-  </si>
-  <si>
     <t>NA</t>
   </si>
   <si>
@@ -103,13 +97,55 @@
   </si>
   <si>
     <t>Restes nids majoritairement sableux</t>
+  </si>
+  <si>
+    <t>Altitude de vol</t>
+  </si>
+  <si>
+    <t>Resolution</t>
+  </si>
+  <si>
+    <t>Surface ortho 2D</t>
+  </si>
+  <si>
+    <t>Surface 2D zone rugosite</t>
+  </si>
+  <si>
+    <t>Surface 3D zone rugosite</t>
+  </si>
+  <si>
+    <t>Lien html</t>
+  </si>
+  <si>
+    <t>pas de modele</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_02/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_03/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_04/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_05/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_06/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_07/App</t>
+  </si>
+  <si>
+    <t>https://www.andromede-ocean3d.com/CARHO/R_PNMCCA_08/App</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +155,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -141,14 +185,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -461,177 +510,296 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D941E263-7268-4471-9E9C-9513FE1DFE1E}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="58" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>149</v>
+        <v>1.81</v>
       </c>
       <c r="C3">
-        <v>187.10599999999999</v>
-      </c>
-      <c r="D3" s="1">
-        <f>C3/B3</f>
-        <v>1.255744966442953</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
+        <v>0.49</v>
+      </c>
+      <c r="D3">
+        <v>249.39</v>
+      </c>
+      <c r="E3">
+        <v>99.89</v>
+      </c>
+      <c r="F3">
+        <v>127.23</v>
+      </c>
+      <c r="G3" s="1">
+        <f>F3/E3</f>
+        <v>1.2737010711782961</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>168</v>
+        <v>1.5</v>
       </c>
       <c r="C4">
-        <v>187.18199999999999</v>
-      </c>
-      <c r="D4" s="1">
-        <f t="shared" ref="D4:D9" si="0">C4/B4</f>
-        <v>1.1141785714285715</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
+        <v>0.40400000000000003</v>
+      </c>
+      <c r="D4">
+        <v>268.39</v>
+      </c>
+      <c r="E4">
+        <v>100.04</v>
+      </c>
+      <c r="F4">
+        <v>110.85</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" ref="G4:G9" si="0">F4/E4</f>
+        <v>1.1080567772890841</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>116</v>
+        <v>1.33</v>
       </c>
       <c r="C5">
-        <v>155.48099999999999</v>
-      </c>
-      <c r="D5" s="1">
+        <v>0.35899999999999999</v>
+      </c>
+      <c r="D5">
+        <v>215.36</v>
+      </c>
+      <c r="E5">
+        <v>99.05</v>
+      </c>
+      <c r="F5">
+        <v>131.49</v>
+      </c>
+      <c r="G5" s="1">
         <f t="shared" si="0"/>
-        <v>1.3403534482758621</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
+        <v>1.3275113579000506</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>156</v>
+        <v>1.43</v>
       </c>
       <c r="C6">
-        <v>233.90899999999999</v>
-      </c>
-      <c r="D6" s="1">
+        <v>0.38200000000000001</v>
+      </c>
+      <c r="D6">
+        <v>257.25</v>
+      </c>
+      <c r="E6">
+        <v>100.47</v>
+      </c>
+      <c r="F6">
+        <v>150.59</v>
+      </c>
+      <c r="G6" s="1">
         <f t="shared" si="0"/>
-        <v>1.4994166666666666</v>
-      </c>
-      <c r="E6" t="s">
-        <v>18</v>
+        <v>1.4988553797153379</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7">
-        <v>118</v>
+        <v>1.22</v>
       </c>
       <c r="C7">
-        <v>135.49299999999999</v>
-      </c>
-      <c r="D7" s="1">
+        <v>0.32800000000000001</v>
+      </c>
+      <c r="D7">
+        <v>218.68</v>
+      </c>
+      <c r="E7">
+        <v>100.26</v>
+      </c>
+      <c r="F7">
+        <v>114.34</v>
+      </c>
+      <c r="G7" s="1">
         <f t="shared" si="0"/>
-        <v>1.1482457627118643</v>
-      </c>
-      <c r="E7" t="s">
-        <v>19</v>
+        <v>1.1404348693397166</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
-        <v>151</v>
+        <v>2.19</v>
       </c>
       <c r="C8">
-        <v>189.14</v>
-      </c>
-      <c r="D8" s="1">
+        <v>0.37</v>
+      </c>
+      <c r="D8">
+        <v>250.83</v>
+      </c>
+      <c r="E8">
+        <v>99.45</v>
+      </c>
+      <c r="F8">
+        <v>123.45</v>
+      </c>
+      <c r="G8" s="1">
         <f t="shared" si="0"/>
-        <v>1.2525827814569535</v>
-      </c>
-      <c r="E8" t="s">
-        <v>20</v>
+        <v>1.2413273001508296</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9">
-        <v>269</v>
+        <v>2.37</v>
       </c>
       <c r="C9">
-        <v>288.55</v>
-      </c>
-      <c r="D9" s="1">
+        <v>0.64100000000000001</v>
+      </c>
+      <c r="D9">
+        <v>369.55</v>
+      </c>
+      <c r="E9">
+        <v>100.1</v>
+      </c>
+      <c r="F9">
+        <v>109.37</v>
+      </c>
+      <c r="G9" s="1">
         <f t="shared" si="0"/>
-        <v>1.0726765799256506</v>
-      </c>
-      <c r="E9" t="s">
-        <v>21</v>
+        <v>1.0926073926073927</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="H3" r:id="rId1" xr:uid="{0587B270-E884-4A15-80E8-A2045BBE88A4}"/>
+    <hyperlink ref="H4" r:id="rId2" xr:uid="{52774D04-F5BD-4F94-BC9D-48043AF59344}"/>
+    <hyperlink ref="H5" r:id="rId3" xr:uid="{CAFE2247-71AA-4EE8-BE50-5C8D4A24C6F5}"/>
+    <hyperlink ref="H6" r:id="rId4" xr:uid="{FE7CF00E-95BC-4D2A-B780-FF7C7C9588F1}"/>
+    <hyperlink ref="H7" r:id="rId5" xr:uid="{6D715105-C566-42F5-8D52-FFAD09214E77}"/>
+    <hyperlink ref="H8" r:id="rId6" xr:uid="{9733F9E4-09CC-40C0-8511-B9A39B1F3837}"/>
+    <hyperlink ref="H9" r:id="rId7" xr:uid="{5C6E9E3B-EE03-4370-B53D-A3A6FBA6D6A0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>